<commit_message>
Add multilingual support (en/hi/hinglish) + meeting link generation
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P9"/>
+  <dimension ref="A1:R9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,6 +497,16 @@
           <t>_row_index</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Meeting Link</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Language</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -552,18 +562,24 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t xml:space="preserve">just the two of us soundsumm tommorow 7 pm and just the 2 of us sounds good for me </t>
+          <t>tomorrow 5pm</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-07-07 20:23:35</t>
+          <t>2026-07-11 18:12:42</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -605,6 +621,12 @@
       <c r="P3" t="n">
         <v>1</v>
       </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -645,6 +667,12 @@
       <c r="P4" t="n">
         <v>2</v>
       </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>hi</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -693,6 +721,12 @@
       <c r="P5" t="n">
         <v>3</v>
       </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -721,17 +755,47 @@
           <t>Pending</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Maybe</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>The user's business has been doing well and they would like to book a meeting for the next day to discuss potential improvements or challenges within their business</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>None specified, but user is looking to discuss business improvements or challenges</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Thank you so far tomorrow, like 7pm's ends perfect for me and I to be honest, want to reduce like the human interaction less, like want to reduce time on data entry and manual things that we can automate. I want to work on that.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>2026-07-11 17:41:42</t>
+        </is>
+      </c>
       <c r="N6" t="inlineStr"/>
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>4</v>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -773,6 +837,12 @@
       <c r="P7" t="n">
         <v>5</v>
       </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -808,7 +878,7 @@
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="b">
+      <c r="N8" t="n">
         <v>1</v>
       </c>
       <c r="O8" t="inlineStr">
@@ -818,6 +888,12 @@
       </c>
       <c r="P8" t="n">
         <v>6</v>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
       </c>
     </row>
     <row r="9">
@@ -859,6 +935,12 @@
       <c r="P9" t="n">
         <v>7</v>
       </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>hinglish</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Fix: lower VAD threshold (500), retry on silence instead of hanging up
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -606,16 +606,40 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+          <t>No Answer</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Not Qualified</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>The user is interested in discussing workflow automation and data synchronization solutions for their business, and is open to exploring options with TechFlow Solutions. The conversation is being conducted in Hindi as per the user's preference. The discussion is in the initial stages, with the assistant introducing the company's services.</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>workflow automation and data synchronization</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>2026-07-11 18:34:24</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">

</xml_diff>

<commit_message>
Switch to English-only: remove Hindi TTS, pure Hindi responses, and language selection prompt
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -648,7 +648,7 @@
       <c r="Q3" t="inlineStr"/>
       <c r="R3" t="inlineStr">
         <is>
-          <t>hinglish</t>
+          <t>en</t>
         </is>
       </c>
     </row>
@@ -694,7 +694,7 @@
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr">
         <is>
-          <t>hi</t>
+          <t>en</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr">
         <is>
-          <t>hinglish</t>
+          <t>en</t>
         </is>
       </c>
     </row>
@@ -864,7 +864,7 @@
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>hinglish</t>
+          <t>en</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       <c r="Q9" t="inlineStr"/>
       <c r="R9" t="inlineStr">
         <is>
-          <t>hinglish</t>
+          <t>en</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix VAD: use avg noise floor, lower threshold to 200, add debug print
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -676,16 +676,32 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
+          <t>No Answer</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Not Qualified</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>The call was initiated by Sarah from TechFlow Solutions, but the conversation did not progress further as there is no response from Mike. The purpose of the call is unknown. No further information is available.</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>2026-07-11 18:47:55</t>
+        </is>
+      </c>
       <c r="N4" t="inlineStr"/>
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
@@ -776,25 +792,29 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>No Answer</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Maybe</t>
+          <t>Not Qualified</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>The user's business has been doing well and they would like to book a meeting for the next day to discuss potential improvements or challenges within their business</t>
+          <t>The conversation just started with a greeting from Sarah from TechFlow Solutions, and no further discussion has taken place. Robert has not responded yet. The purpose of the call is not yet clear.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>None specified, but user is looking to discuss business improvements or challenges</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>none</t>
@@ -807,7 +827,7 @@
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>2026-07-11 17:41:42</t>
+          <t>2026-07-11 18:48:14</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>

</xml_diff>

<commit_message>
Simplify mic: record 6s flat, no VAD, no calibration
</commit_message>
<xml_diff>
--- a/data/leads.xlsx
+++ b/data/leads.xlsx
@@ -866,16 +866,40 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+          <t>No Answer</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Not Qualified</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>The conversation just started with an introduction from Sarah from TechFlow Solutions to Lisa, and no discussion has taken place yet. The purpose of the call is not yet known. The conversation has not progressed beyond the initial greeting.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2026-07-11 18:49:26</t>
+        </is>
+      </c>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">

</xml_diff>